<commit_message>
I populated the parameter arrays and added parameter values taken from v.1 spreadsheet
</commit_message>
<xml_diff>
--- a/Parameter_valuesV.1.xlsx
+++ b/Parameter_valuesV.1.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/oliviaaguiar/Desktop/Dissertation/SIS_model/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E67494DC-3F0C-8546-9983-CF8442EDBB0E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A4B89F87-FDE5-AD46-8668-F1BFCC8942D4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28800" yWindow="0" windowWidth="28800" windowHeight="18000" xr2:uid="{C0207AB7-C4D1-5541-A64D-9885F356C8AB}"/>
   </bookViews>
@@ -43,6 +43,7 @@
     <author>tc={ED84AEA7-AFB5-EA49-88BC-F2FB8656F9D5}</author>
     <author>tc={0E431F38-632E-5648-9E07-E7E0D238639C}</author>
     <author>tc={8E54BFB9-3CC5-7748-BE5A-75057D53EA6B}</author>
+    <author>tc={34A2E183-AC07-454E-9CA3-9D4C9D1132CD}</author>
     <author>tc={A44ED92B-2083-AF47-8C20-4D773F054C03}</author>
   </authors>
   <commentList>
@@ -88,7 +89,17 @@
     taken by dividing 1 by the number of weeks where birth occurs multiplied by random number in range of overall birth rate</t>
       </text>
     </comment>
-    <comment ref="C20" authorId="5" shapeId="0" xr:uid="{A44ED92B-2083-AF47-8C20-4D773F054C03}">
+    <comment ref="K1" authorId="5" shapeId="0" xr:uid="{34A2E183-AC07-454E-9CA3-9D4C9D1132CD}">
+      <text>
+        <t>[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    keeping this the same for all classes for now
+Reply:
+    taken again like the virulence calculation, 15-30% yearly then multiplied</t>
+      </text>
+    </comment>
+    <comment ref="C20" authorId="6" shapeId="0" xr:uid="{A44ED92B-2083-AF47-8C20-4D773F054C03}">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -101,7 +112,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="145" uniqueCount="70">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="198" uniqueCount="72">
   <si>
     <t>Date</t>
   </si>
@@ -311,6 +322,12 @@
   </si>
   <si>
     <t>1/[13*50~90)]</t>
+  </si>
+  <si>
+    <t>Natural death (mu)</t>
+  </si>
+  <si>
+    <t>1/[52*(15~30)]</t>
   </si>
 </sst>
 </file>
@@ -713,6 +730,12 @@
   <threadedComment ref="I1" dT="2026-06-24T16:29:57.00" personId="{4162FE76-C56F-5A4F-B5CA-CB15DF8228F5}" id="{8BDB10BE-11DC-F54E-9ACA-1760299E6B48}" parentId="{8E54BFB9-3CC5-7748-BE5A-75057D53EA6B}">
     <text>taken by dividing 1 by the number of weeks where birth occurs multiplied by random number in range of overall birth rate</text>
   </threadedComment>
+  <threadedComment ref="K1" dT="2026-06-24T16:35:01.28" personId="{4162FE76-C56F-5A4F-B5CA-CB15DF8228F5}" id="{34A2E183-AC07-454E-9CA3-9D4C9D1132CD}">
+    <text>keeping this the same for all classes for now</text>
+  </threadedComment>
+  <threadedComment ref="K1" dT="2026-06-24T16:41:37.29" personId="{4162FE76-C56F-5A4F-B5CA-CB15DF8228F5}" id="{E9EF0372-DBF9-3D45-9428-6C1AE218BBD0}" parentId="{34A2E183-AC07-454E-9CA3-9D4C9D1132CD}">
+    <text>taken again like the virulence calculation, 15-30% yearly then multiplied</text>
+  </threadedComment>
   <threadedComment ref="C20" dT="2026-06-24T15:57:34.84" personId="{4162FE76-C56F-5A4F-B5CA-CB15DF8228F5}" id="{A44ED92B-2083-AF47-8C20-4D773F054C03}">
     <text>MYLU infection to 100% by Jan according to http://dx.doi.org/10.1098/rspb.2014.2335</text>
     <extLst>
@@ -727,7 +750,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9A1AEC79-FE41-444E-A91D-AFDB48402896}">
-  <dimension ref="A1:J53"/>
+  <dimension ref="A1:K53"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="3" max="3" width="27.33203125" bestFit="1" customWidth="1"/>
@@ -739,7 +762,7 @@
     <col min="10" max="10" width="13.33203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -770,8 +793,11 @@
       <c r="J1" t="s">
         <v>66</v>
       </c>
-    </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K1" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="2" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>2</v>
       </c>
@@ -802,8 +828,11 @@
       <c r="J2">
         <v>0</v>
       </c>
-    </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K2" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="3" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>4</v>
       </c>
@@ -834,8 +863,11 @@
       <c r="J3">
         <v>0</v>
       </c>
-    </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K3" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="4" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>5</v>
       </c>
@@ -866,8 +898,11 @@
       <c r="J4">
         <v>0</v>
       </c>
-    </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K4" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="5" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>6</v>
       </c>
@@ -898,8 +933,11 @@
       <c r="J5">
         <v>0</v>
       </c>
-    </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K5" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="6" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
         <v>7</v>
       </c>
@@ -930,8 +968,11 @@
       <c r="J6">
         <v>0</v>
       </c>
-    </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K6" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="7" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
         <v>8</v>
       </c>
@@ -962,8 +1003,11 @@
       <c r="J7">
         <v>0</v>
       </c>
-    </row>
-    <row r="8" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K7" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="8" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
         <v>9</v>
       </c>
@@ -994,8 +1038,11 @@
       <c r="J8">
         <v>0</v>
       </c>
-    </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K8" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="9" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
         <v>10</v>
       </c>
@@ -1026,8 +1073,11 @@
       <c r="J9">
         <v>0</v>
       </c>
-    </row>
-    <row r="10" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K9" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="10" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
         <v>11</v>
       </c>
@@ -1058,8 +1108,11 @@
       <c r="J10">
         <v>0</v>
       </c>
-    </row>
-    <row r="11" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K10" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="11" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
         <v>12</v>
       </c>
@@ -1090,8 +1143,11 @@
       <c r="J11">
         <v>0</v>
       </c>
-    </row>
-    <row r="12" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K11" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="12" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
         <v>13</v>
       </c>
@@ -1122,8 +1178,11 @@
       <c r="J12">
         <v>0</v>
       </c>
-    </row>
-    <row r="13" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K12" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="13" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
         <v>14</v>
       </c>
@@ -1154,8 +1213,11 @@
       <c r="J13">
         <v>0</v>
       </c>
-    </row>
-    <row r="14" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K13" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="14" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
         <v>15</v>
       </c>
@@ -1186,8 +1248,11 @@
       <c r="J14">
         <v>0</v>
       </c>
-    </row>
-    <row r="15" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K14" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="15" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
         <v>16</v>
       </c>
@@ -1218,8 +1283,11 @@
       <c r="J15">
         <v>0</v>
       </c>
-    </row>
-    <row r="16" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K15" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="16" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
         <v>17</v>
       </c>
@@ -1250,8 +1318,11 @@
       <c r="J16">
         <v>0</v>
       </c>
-    </row>
-    <row r="17" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K16" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="17" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
         <v>18</v>
       </c>
@@ -1282,8 +1353,11 @@
       <c r="J17">
         <v>0</v>
       </c>
-    </row>
-    <row r="18" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K17" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="18" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
         <v>19</v>
       </c>
@@ -1314,8 +1388,11 @@
       <c r="J18">
         <v>0</v>
       </c>
-    </row>
-    <row r="19" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K18" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="19" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
         <v>20</v>
       </c>
@@ -1346,8 +1423,11 @@
       <c r="J19">
         <v>0</v>
       </c>
-    </row>
-    <row r="20" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K19" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="20" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
         <v>21</v>
       </c>
@@ -1378,8 +1458,11 @@
       <c r="J20">
         <v>0</v>
       </c>
-    </row>
-    <row r="21" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K20" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="21" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
         <v>22</v>
       </c>
@@ -1410,8 +1493,11 @@
       <c r="J21">
         <v>0</v>
       </c>
-    </row>
-    <row r="22" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K21" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="22" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
         <v>23</v>
       </c>
@@ -1442,8 +1528,11 @@
       <c r="J22">
         <v>0</v>
       </c>
-    </row>
-    <row r="23" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K22" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="23" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A23" t="s">
         <v>24</v>
       </c>
@@ -1474,8 +1563,11 @@
       <c r="J23">
         <v>0</v>
       </c>
-    </row>
-    <row r="24" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K23" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="24" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A24" t="s">
         <v>25</v>
       </c>
@@ -1506,8 +1598,11 @@
       <c r="J24">
         <v>0</v>
       </c>
-    </row>
-    <row r="25" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K24" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="25" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A25" t="s">
         <v>26</v>
       </c>
@@ -1538,8 +1633,11 @@
       <c r="J25">
         <v>0</v>
       </c>
-    </row>
-    <row r="26" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K25" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="26" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A26" t="s">
         <v>27</v>
       </c>
@@ -1570,8 +1668,11 @@
       <c r="J26">
         <v>0</v>
       </c>
-    </row>
-    <row r="27" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K26" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="27" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A27" t="s">
         <v>28</v>
       </c>
@@ -1602,8 +1703,11 @@
       <c r="J27">
         <v>0</v>
       </c>
-    </row>
-    <row r="28" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K27" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="28" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A28" t="s">
         <v>29</v>
       </c>
@@ -1634,8 +1738,11 @@
       <c r="J28">
         <v>0</v>
       </c>
-    </row>
-    <row r="29" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K28" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="29" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A29" t="s">
         <v>30</v>
       </c>
@@ -1666,8 +1773,11 @@
       <c r="J29">
         <v>0</v>
       </c>
-    </row>
-    <row r="30" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K29" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="30" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A30" t="s">
         <v>31</v>
       </c>
@@ -1698,8 +1808,11 @@
       <c r="J30">
         <v>0</v>
       </c>
-    </row>
-    <row r="31" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K30" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="31" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A31" t="s">
         <v>32</v>
       </c>
@@ -1730,8 +1843,11 @@
       <c r="J31">
         <v>0</v>
       </c>
-    </row>
-    <row r="32" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K31" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="32" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A32" t="s">
         <v>33</v>
       </c>
@@ -1762,8 +1878,11 @@
       <c r="J32">
         <v>0</v>
       </c>
-    </row>
-    <row r="33" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K32" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="33" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A33" t="s">
         <v>34</v>
       </c>
@@ -1794,8 +1913,11 @@
       <c r="J33">
         <v>0</v>
       </c>
-    </row>
-    <row r="34" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K33" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="34" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A34" t="s">
         <v>35</v>
       </c>
@@ -1826,8 +1948,11 @@
       <c r="J34">
         <v>0</v>
       </c>
-    </row>
-    <row r="35" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K34" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="35" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A35" t="s">
         <v>36</v>
       </c>
@@ -1858,8 +1983,11 @@
       <c r="J35">
         <v>0</v>
       </c>
-    </row>
-    <row r="36" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K35" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="36" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A36" t="s">
         <v>37</v>
       </c>
@@ -1890,8 +2018,11 @@
       <c r="J36">
         <v>0</v>
       </c>
-    </row>
-    <row r="37" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K36" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="37" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A37" t="s">
         <v>38</v>
       </c>
@@ -1922,8 +2053,11 @@
       <c r="J37">
         <v>0</v>
       </c>
-    </row>
-    <row r="38" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K37" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="38" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A38" t="s">
         <v>39</v>
       </c>
@@ -1954,8 +2088,11 @@
       <c r="J38">
         <v>0</v>
       </c>
-    </row>
-    <row r="39" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K38" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="39" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A39" t="s">
         <v>40</v>
       </c>
@@ -1986,8 +2123,11 @@
       <c r="J39">
         <v>0</v>
       </c>
-    </row>
-    <row r="40" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K39" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="40" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A40" t="s">
         <v>41</v>
       </c>
@@ -2018,8 +2158,11 @@
       <c r="J40">
         <v>0</v>
       </c>
-    </row>
-    <row r="41" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K40" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="41" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A41" t="s">
         <v>42</v>
       </c>
@@ -2050,8 +2193,11 @@
       <c r="J41">
         <v>0</v>
       </c>
-    </row>
-    <row r="42" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K41" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="42" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A42" t="s">
         <v>43</v>
       </c>
@@ -2082,8 +2228,11 @@
       <c r="J42">
         <v>0</v>
       </c>
-    </row>
-    <row r="43" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K42" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="43" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A43" t="s">
         <v>44</v>
       </c>
@@ -2114,8 +2263,11 @@
       <c r="J43">
         <v>0</v>
       </c>
-    </row>
-    <row r="44" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K43" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="44" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A44" t="s">
         <v>45</v>
       </c>
@@ -2146,8 +2298,11 @@
       <c r="J44">
         <v>0</v>
       </c>
-    </row>
-    <row r="45" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K44" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="45" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A45" t="s">
         <v>46</v>
       </c>
@@ -2178,8 +2333,11 @@
       <c r="J45" t="s">
         <v>67</v>
       </c>
-    </row>
-    <row r="46" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K45" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="46" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A46" t="s">
         <v>47</v>
       </c>
@@ -2210,8 +2368,11 @@
       <c r="J46" t="s">
         <v>67</v>
       </c>
-    </row>
-    <row r="47" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K46" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="47" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A47" t="s">
         <v>48</v>
       </c>
@@ -2242,8 +2403,11 @@
       <c r="J47" t="s">
         <v>67</v>
       </c>
-    </row>
-    <row r="48" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K47" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="48" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A48" t="s">
         <v>49</v>
       </c>
@@ -2274,8 +2438,11 @@
       <c r="J48" t="s">
         <v>67</v>
       </c>
-    </row>
-    <row r="49" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K48" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="49" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A49" t="s">
         <v>50</v>
       </c>
@@ -2306,8 +2473,11 @@
       <c r="J49" t="s">
         <v>67</v>
       </c>
-    </row>
-    <row r="50" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K49" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="50" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A50" t="s">
         <v>51</v>
       </c>
@@ -2338,8 +2508,11 @@
       <c r="J50" t="s">
         <v>67</v>
       </c>
-    </row>
-    <row r="51" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K50" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="51" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A51" t="s">
         <v>52</v>
       </c>
@@ -2370,8 +2543,11 @@
       <c r="J51" t="s">
         <v>67</v>
       </c>
-    </row>
-    <row r="52" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K51" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="52" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A52" t="s">
         <v>53</v>
       </c>
@@ -2402,8 +2578,11 @@
       <c r="J52" t="s">
         <v>67</v>
       </c>
-    </row>
-    <row r="53" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K52" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="53" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A53" t="s">
         <v>54</v>
       </c>
@@ -2433,6 +2612,9 @@
       </c>
       <c r="J53" t="s">
         <v>67</v>
+      </c>
+      <c r="K53" t="s">
+        <v>71</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
made changes to virulence and birth fractions
</commit_message>
<xml_diff>
--- a/Parameter_valuesV.1.xlsx
+++ b/Parameter_valuesV.1.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/oliviaaguiar/Desktop/Dissertation/SIS_model/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A4B89F87-FDE5-AD46-8668-F1BFCC8942D4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{901DE66D-F3AE-534F-B718-94030400F9E3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28800" yWindow="0" windowWidth="28800" windowHeight="18000" xr2:uid="{C0207AB7-C4D1-5541-A64D-9885F356C8AB}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="38400" windowHeight="21600" xr2:uid="{C0207AB7-C4D1-5541-A64D-9885F356C8AB}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>

</xml_diff>

<commit_message>
changed beta to a constant number, because transmission is determined by the number of bats in the hibernacula, so our parameters with hibernation immergence take care of that part of the model
made some changes to the function and started a for loop to test out the model function
</commit_message>
<xml_diff>
--- a/Parameter_valuesV.1.xlsx
+++ b/Parameter_valuesV.1.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/oliviaaguiar/Desktop/Dissertation/SIS_model/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{901DE66D-F3AE-534F-B718-94030400F9E3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D08765A3-3044-C64F-B1F5-060C2B5E4209}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="38400" windowHeight="21600" xr2:uid="{C0207AB7-C4D1-5541-A64D-9885F356C8AB}"/>
   </bookViews>
@@ -40,14 +40,13 @@
   <authors>
     <author>tc={30895D16-7676-BA44-990B-B127DB724EBD}</author>
     <author>tc={BC4039C5-1ECF-E04B-85F4-3493754D8932}</author>
-    <author>tc={ED84AEA7-AFB5-EA49-88BC-F2FB8656F9D5}</author>
+    <author>tc={BF579079-8378-8948-A692-C6847AAF6B70}</author>
     <author>tc={0E431F38-632E-5648-9E07-E7E0D238639C}</author>
-    <author>tc={8E54BFB9-3CC5-7748-BE5A-75057D53EA6B}</author>
-    <author>tc={34A2E183-AC07-454E-9CA3-9D4C9D1132CD}</author>
+    <author>tc={F3259CE0-1A3C-5A4A-91DB-834F36616FC8}</author>
     <author>tc={A44ED92B-2083-AF47-8C20-4D773F054C03}</author>
   </authors>
   <commentList>
-    <comment ref="D1" authorId="0" shapeId="0" xr:uid="{30895D16-7676-BA44-990B-B127DB724EBD}">
+    <comment ref="D2" authorId="0" shapeId="0" xr:uid="{30895D16-7676-BA44-990B-B127DB724EBD}">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -55,7 +54,7 @@
     7 week span to enter hibernation, values of h are 1/7 then in the final week is 1 to get all bats to move to hibernation</t>
       </text>
     </comment>
-    <comment ref="F1" authorId="1" shapeId="0" xr:uid="{BC4039C5-1ECF-E04B-85F4-3493754D8932}">
+    <comment ref="F2" authorId="1" shapeId="0" xr:uid="{BC4039C5-1ECF-E04B-85F4-3493754D8932}">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -63,15 +62,15 @@
     these values estimated the same way as immergence- prevalence for MYLU to 100% by January (8 week period) so used 1/8 for each week and 1 in the final week so all become infected</t>
       </text>
     </comment>
-    <comment ref="G1" authorId="2" shapeId="0" xr:uid="{ED84AEA7-AFB5-EA49-88BC-F2FB8656F9D5}">
+    <comment ref="G2" authorId="2" shapeId="0" xr:uid="{BF579079-8378-8948-A692-C6847AAF6B70}">
       <text>
-        <t xml:space="preserve">[Threaded comment]
+        <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
 Comment:
-    estimated by taking the weeks where death occurs (13) and multiply by a random no. from 50-90 (overall virulence est.) </t>
+    for now it is calculated from overall 70% death rate from WNS, see notes from 6/24- is 0.0885</t>
       </text>
     </comment>
-    <comment ref="H1" authorId="3" shapeId="0" xr:uid="{0E431F38-632E-5648-9E07-E7E0D238639C}">
+    <comment ref="H2" authorId="3" shapeId="0" xr:uid="{0E431F38-632E-5648-9E07-E7E0D238639C}">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -79,27 +78,15 @@
     Also estimated like immergence- if you survive then you clear infection in four weeks so 1/4 and then in final week its 1 so all bats recover</t>
       </text>
     </comment>
-    <comment ref="I1" authorId="4" shapeId="0" xr:uid="{8E54BFB9-3CC5-7748-BE5A-75057D53EA6B}">
+    <comment ref="K2" authorId="4" shapeId="0" xr:uid="{F3259CE0-1A3C-5A4A-91DB-834F36616FC8}">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
 Comment:
-    birth yearling and adult is the same for now
-Reply:
-    taken by dividing 1 by the number of weeks where birth occurs multiplied by random number in range of overall birth rate</t>
+    taken from average 30 year lifespan</t>
       </text>
     </comment>
-    <comment ref="K1" authorId="5" shapeId="0" xr:uid="{34A2E183-AC07-454E-9CA3-9D4C9D1132CD}">
-      <text>
-        <t>[Threaded comment]
-Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
-Comment:
-    keeping this the same for all classes for now
-Reply:
-    taken again like the virulence calculation, 15-30% yearly then multiplied</t>
-      </text>
-    </comment>
-    <comment ref="C20" authorId="6" shapeId="0" xr:uid="{A44ED92B-2083-AF47-8C20-4D773F054C03}">
+    <comment ref="C21" authorId="5" shapeId="0" xr:uid="{A44ED92B-2083-AF47-8C20-4D773F054C03}">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -112,7 +99,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="198" uniqueCount="72">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="174" uniqueCount="77">
   <si>
     <t>Date</t>
   </si>
@@ -315,38 +302,47 @@
     <t>Birth adult (b2)</t>
   </si>
   <si>
-    <t>1/[9*(70~100)]</t>
-  </si>
-  <si>
     <t>Emmergence (e)</t>
   </si>
   <si>
-    <t>1/[13*50~90)]</t>
-  </si>
-  <si>
     <t>Natural death (mu)</t>
   </si>
   <si>
-    <t>1/[52*(15~30)]</t>
+    <t xml:space="preserve">this is a weekly death fraction for hibernating individuals that are infected with WNS </t>
+  </si>
+  <si>
+    <t>1/(30*52)</t>
+  </si>
+  <si>
+    <t>this is a weekly recovery fraction for individuals infected with WNS</t>
+  </si>
+  <si>
+    <t>this is a weekly infection transmission fraction</t>
+  </si>
+  <si>
+    <t>this is a weekly emmergence fraction</t>
+  </si>
+  <si>
+    <t>this is a weekly immergence fraction</t>
+  </si>
+  <si>
+    <t>this is a weekly birth fraction</t>
+  </si>
+  <si>
+    <t>this is a weekly natural death fraction</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="1" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <color rgb="FF000000"/>
-      <name val="Tahoma"/>
-      <family val="2"/>
     </font>
   </fonts>
   <fills count="2">
@@ -712,31 +708,22 @@
 
 <file path=xl/threadedComments/threadedComment1.xml><?xml version="1.0" encoding="utf-8"?>
 <ThreadedComments xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <threadedComment ref="D1" dT="2026-06-24T15:56:53.29" personId="{4162FE76-C56F-5A4F-B5CA-CB15DF8228F5}" id="{30895D16-7676-BA44-990B-B127DB724EBD}">
+  <threadedComment ref="D2" dT="2026-06-24T15:56:53.29" personId="{4162FE76-C56F-5A4F-B5CA-CB15DF8228F5}" id="{30895D16-7676-BA44-990B-B127DB724EBD}">
     <text>7 week span to enter hibernation, values of h are 1/7 then in the final week is 1 to get all bats to move to hibernation</text>
   </threadedComment>
-  <threadedComment ref="F1" dT="2026-06-24T15:59:34.37" personId="{4162FE76-C56F-5A4F-B5CA-CB15DF8228F5}" id="{BC4039C5-1ECF-E04B-85F4-3493754D8932}">
+  <threadedComment ref="F2" dT="2026-06-24T15:59:34.37" personId="{4162FE76-C56F-5A4F-B5CA-CB15DF8228F5}" id="{BC4039C5-1ECF-E04B-85F4-3493754D8932}">
     <text>these values estimated the same way as immergence- prevalence for MYLU to 100% by January (8 week period) so used 1/8 for each week and 1 in the final week so all become infected</text>
   </threadedComment>
-  <threadedComment ref="G1" dT="2026-06-24T16:29:08.90" personId="{4162FE76-C56F-5A4F-B5CA-CB15DF8228F5}" id="{ED84AEA7-AFB5-EA49-88BC-F2FB8656F9D5}">
-    <text xml:space="preserve">estimated by taking the weeks where death occurs (13) and multiply by a random no. from 50-90 (overall virulence est.) </text>
+  <threadedComment ref="G2" dT="2026-06-24T17:30:11.52" personId="{4162FE76-C56F-5A4F-B5CA-CB15DF8228F5}" id="{BF579079-8378-8948-A692-C6847AAF6B70}">
+    <text>for now it is calculated from overall 70% death rate from WNS, see notes from 6/24- is 0.0885</text>
   </threadedComment>
-  <threadedComment ref="H1" dT="2026-06-24T16:04:49.89" personId="{4162FE76-C56F-5A4F-B5CA-CB15DF8228F5}" id="{0E431F38-632E-5648-9E07-E7E0D238639C}">
+  <threadedComment ref="H2" dT="2026-06-24T16:04:49.89" personId="{4162FE76-C56F-5A4F-B5CA-CB15DF8228F5}" id="{0E431F38-632E-5648-9E07-E7E0D238639C}">
     <text>Also estimated like immergence- if you survive then you clear infection in four weeks so 1/4 and then in final week its 1 so all bats recover</text>
   </threadedComment>
-  <threadedComment ref="I1" dT="2026-06-24T16:10:40.55" personId="{4162FE76-C56F-5A4F-B5CA-CB15DF8228F5}" id="{8E54BFB9-3CC5-7748-BE5A-75057D53EA6B}">
-    <text>birth yearling and adult is the same for now</text>
+  <threadedComment ref="K2" dT="2026-06-24T17:38:37.37" personId="{4162FE76-C56F-5A4F-B5CA-CB15DF8228F5}" id="{F3259CE0-1A3C-5A4A-91DB-834F36616FC8}">
+    <text>taken from average 30 year lifespan</text>
   </threadedComment>
-  <threadedComment ref="I1" dT="2026-06-24T16:29:57.00" personId="{4162FE76-C56F-5A4F-B5CA-CB15DF8228F5}" id="{8BDB10BE-11DC-F54E-9ACA-1760299E6B48}" parentId="{8E54BFB9-3CC5-7748-BE5A-75057D53EA6B}">
-    <text>taken by dividing 1 by the number of weeks where birth occurs multiplied by random number in range of overall birth rate</text>
-  </threadedComment>
-  <threadedComment ref="K1" dT="2026-06-24T16:35:01.28" personId="{4162FE76-C56F-5A4F-B5CA-CB15DF8228F5}" id="{34A2E183-AC07-454E-9CA3-9D4C9D1132CD}">
-    <text>keeping this the same for all classes for now</text>
-  </threadedComment>
-  <threadedComment ref="K1" dT="2026-06-24T16:41:37.29" personId="{4162FE76-C56F-5A4F-B5CA-CB15DF8228F5}" id="{E9EF0372-DBF9-3D45-9428-6C1AE218BBD0}" parentId="{34A2E183-AC07-454E-9CA3-9D4C9D1132CD}">
-    <text>taken again like the virulence calculation, 15-30% yearly then multiplied</text>
-  </threadedComment>
-  <threadedComment ref="C20" dT="2026-06-24T15:57:34.84" personId="{4162FE76-C56F-5A4F-B5CA-CB15DF8228F5}" id="{A44ED92B-2083-AF47-8C20-4D773F054C03}">
+  <threadedComment ref="C21" dT="2026-06-24T15:57:34.84" personId="{4162FE76-C56F-5A4F-B5CA-CB15DF8228F5}" id="{A44ED92B-2083-AF47-8C20-4D773F054C03}">
     <text>MYLU infection to 100% by Jan according to http://dx.doi.org/10.1098/rspb.2014.2335</text>
     <extLst>
       <x:ext xmlns:xltc2="http://schemas.microsoft.com/office/spreadsheetml/2020/threadedcomments2" uri="{F7C98A9C-CBB3-438F-8F68-D28B6AF4A901}">
@@ -750,7 +737,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9A1AEC79-FE41-444E-A91D-AFDB48402896}">
-  <dimension ref="A1:K53"/>
+  <dimension ref="A1:K54"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="3" max="3" width="27.33203125" bestFit="1" customWidth="1"/>
@@ -762,82 +749,70 @@
     <col min="10" max="10" width="13.33203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" t="s">
-        <v>3</v>
-      </c>
+    <row r="1" spans="1:11" ht="98" customHeight="1" x14ac:dyDescent="0.2">
       <c r="D1" s="1" t="s">
-        <v>61</v>
+        <v>74</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>68</v>
+        <v>73</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>62</v>
+        <v>72</v>
       </c>
       <c r="G1" t="s">
-        <v>63</v>
+        <v>69</v>
       </c>
       <c r="H1" t="s">
-        <v>64</v>
-      </c>
-      <c r="I1" t="s">
-        <v>65</v>
-      </c>
-      <c r="J1" t="s">
-        <v>66</v>
+        <v>71</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>75</v>
       </c>
       <c r="K1" t="s">
-        <v>70</v>
+        <v>76</v>
       </c>
     </row>
     <row r="2" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
-        <v>2</v>
-      </c>
-      <c r="B2">
+        <v>0</v>
+      </c>
+      <c r="B2" t="s">
         <v>1</v>
       </c>
       <c r="C2" t="s">
-        <v>55</v>
-      </c>
-      <c r="D2" s="1">
-        <v>0</v>
-      </c>
-      <c r="E2" s="1">
-        <v>0</v>
-      </c>
-      <c r="F2" s="1">
-        <v>0</v>
-      </c>
-      <c r="G2">
-        <v>0</v>
-      </c>
-      <c r="H2">
-        <v>0</v>
-      </c>
-      <c r="I2">
-        <v>0</v>
-      </c>
-      <c r="J2">
-        <v>0</v>
+        <v>3</v>
+      </c>
+      <c r="D2" s="1" t="s">
+        <v>61</v>
+      </c>
+      <c r="E2" s="1" t="s">
+        <v>67</v>
+      </c>
+      <c r="F2" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="G2" t="s">
+        <v>63</v>
+      </c>
+      <c r="H2" t="s">
+        <v>64</v>
+      </c>
+      <c r="I2" t="s">
+        <v>65</v>
+      </c>
+      <c r="J2" t="s">
+        <v>66</v>
       </c>
       <c r="K2" t="s">
-        <v>71</v>
+        <v>68</v>
       </c>
     </row>
     <row r="3" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="B3">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C3" t="s">
         <v>55</v>
@@ -849,7 +824,7 @@
         <v>0</v>
       </c>
       <c r="F3" s="1">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="G3">
         <v>0</v>
@@ -864,15 +839,15 @@
         <v>0</v>
       </c>
       <c r="K3" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
     </row>
     <row r="4" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B4">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C4" t="s">
         <v>55</v>
@@ -884,7 +859,7 @@
         <v>0</v>
       </c>
       <c r="F4" s="1">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="G4">
         <v>0</v>
@@ -899,15 +874,15 @@
         <v>0</v>
       </c>
       <c r="K4" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
     </row>
     <row r="5" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B5">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C5" t="s">
         <v>55</v>
@@ -919,7 +894,7 @@
         <v>0</v>
       </c>
       <c r="F5" s="1">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="G5">
         <v>0</v>
@@ -934,15 +909,15 @@
         <v>0</v>
       </c>
       <c r="K5" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
     </row>
     <row r="6" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B6">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C6" t="s">
         <v>55</v>
@@ -954,7 +929,7 @@
         <v>0</v>
       </c>
       <c r="F6" s="1">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="G6">
         <v>0</v>
@@ -969,15 +944,15 @@
         <v>0</v>
       </c>
       <c r="K6" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
     </row>
     <row r="7" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B7">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="C7" t="s">
         <v>55</v>
@@ -989,7 +964,7 @@
         <v>0</v>
       </c>
       <c r="F7" s="1">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="G7">
         <v>0</v>
@@ -1004,15 +979,15 @@
         <v>0</v>
       </c>
       <c r="K7" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
     </row>
     <row r="8" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B8">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="C8" t="s">
         <v>55</v>
@@ -1024,7 +999,7 @@
         <v>0</v>
       </c>
       <c r="F8" s="1">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="G8">
         <v>0</v>
@@ -1039,15 +1014,15 @@
         <v>0</v>
       </c>
       <c r="K8" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
     </row>
     <row r="9" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B9">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="C9" t="s">
         <v>55</v>
@@ -1059,7 +1034,7 @@
         <v>0</v>
       </c>
       <c r="F9" s="1">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="G9">
         <v>0</v>
@@ -1074,15 +1049,15 @@
         <v>0</v>
       </c>
       <c r="K9" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
     </row>
     <row r="10" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B10">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="C10" t="s">
         <v>55</v>
@@ -1094,7 +1069,7 @@
         <v>0</v>
       </c>
       <c r="F10" s="1">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="G10">
         <v>0</v>
@@ -1109,15 +1084,15 @@
         <v>0</v>
       </c>
       <c r="K10" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
     </row>
     <row r="11" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B11">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="C11" t="s">
         <v>55</v>
@@ -1129,7 +1104,7 @@
         <v>0</v>
       </c>
       <c r="F11" s="1">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="G11">
         <v>0</v>
@@ -1144,15 +1119,15 @@
         <v>0</v>
       </c>
       <c r="K11" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
     </row>
     <row r="12" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B12">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="C12" t="s">
         <v>55</v>
@@ -1164,7 +1139,7 @@
         <v>0</v>
       </c>
       <c r="F12" s="1">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="G12">
         <v>0</v>
@@ -1179,27 +1154,27 @@
         <v>0</v>
       </c>
       <c r="K12" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
     </row>
     <row r="13" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B13">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C13" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="D13" s="1">
-        <v>0.14285714285714285</v>
+        <v>0</v>
       </c>
       <c r="E13" s="1">
         <v>0</v>
       </c>
       <c r="F13" s="1">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="G13">
         <v>0</v>
@@ -1214,15 +1189,15 @@
         <v>0</v>
       </c>
       <c r="K13" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
     </row>
     <row r="14" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B14">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C14" t="s">
         <v>56</v>
@@ -1234,7 +1209,7 @@
         <v>0</v>
       </c>
       <c r="F14" s="1">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="G14">
         <v>0</v>
@@ -1249,15 +1224,15 @@
         <v>0</v>
       </c>
       <c r="K14" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
     </row>
     <row r="15" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B15">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C15" t="s">
         <v>56</v>
@@ -1269,7 +1244,7 @@
         <v>0</v>
       </c>
       <c r="F15" s="1">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="G15">
         <v>0</v>
@@ -1284,15 +1259,15 @@
         <v>0</v>
       </c>
       <c r="K15" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
     </row>
     <row r="16" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B16">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C16" t="s">
         <v>56</v>
@@ -1304,7 +1279,7 @@
         <v>0</v>
       </c>
       <c r="F16" s="1">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="G16">
         <v>0</v>
@@ -1319,15 +1294,15 @@
         <v>0</v>
       </c>
       <c r="K16" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
     </row>
     <row r="17" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B17">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="C17" t="s">
         <v>56</v>
@@ -1339,7 +1314,7 @@
         <v>0</v>
       </c>
       <c r="F17" s="1">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="G17">
         <v>0</v>
@@ -1354,15 +1329,15 @@
         <v>0</v>
       </c>
       <c r="K17" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
     </row>
     <row r="18" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B18">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="C18" t="s">
         <v>56</v>
@@ -1374,7 +1349,7 @@
         <v>0</v>
       </c>
       <c r="F18" s="1">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="G18">
         <v>0</v>
@@ -1389,27 +1364,27 @@
         <v>0</v>
       </c>
       <c r="K18" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
     </row>
     <row r="19" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B19">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C19" t="s">
         <v>56</v>
       </c>
       <c r="D19" s="1">
-        <v>1</v>
+        <v>0.14285714285714285</v>
       </c>
       <c r="E19" s="1">
         <v>0</v>
       </c>
       <c r="F19" s="1">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="G19">
         <v>0</v>
@@ -1424,27 +1399,27 @@
         <v>0</v>
       </c>
       <c r="K19" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
     </row>
     <row r="20" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B20">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C20" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="D20" s="1">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E20" s="1">
         <v>0</v>
       </c>
       <c r="F20" s="1">
-        <v>0.125</v>
+        <v>0.5</v>
       </c>
       <c r="G20">
         <v>0</v>
@@ -1459,15 +1434,15 @@
         <v>0</v>
       </c>
       <c r="K20" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
     </row>
     <row r="21" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B21">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="C21" t="s">
         <v>57</v>
@@ -1479,7 +1454,7 @@
         <v>0</v>
       </c>
       <c r="F21" s="1">
-        <v>0.125</v>
+        <v>0.5</v>
       </c>
       <c r="G21">
         <v>0</v>
@@ -1494,15 +1469,15 @@
         <v>0</v>
       </c>
       <c r="K21" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
     </row>
     <row r="22" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B22">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="C22" t="s">
         <v>57</v>
@@ -1514,7 +1489,7 @@
         <v>0</v>
       </c>
       <c r="F22" s="1">
-        <v>0.125</v>
+        <v>0.5</v>
       </c>
       <c r="G22">
         <v>0</v>
@@ -1529,15 +1504,15 @@
         <v>0</v>
       </c>
       <c r="K22" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
     </row>
     <row r="23" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A23" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B23">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="C23" t="s">
         <v>57</v>
@@ -1549,7 +1524,7 @@
         <v>0</v>
       </c>
       <c r="F23" s="1">
-        <v>0.125</v>
+        <v>0.5</v>
       </c>
       <c r="G23">
         <v>0</v>
@@ -1564,15 +1539,15 @@
         <v>0</v>
       </c>
       <c r="K23" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
     </row>
     <row r="24" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A24" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="B24">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="C24" t="s">
         <v>57</v>
@@ -1584,7 +1559,7 @@
         <v>0</v>
       </c>
       <c r="F24" s="1">
-        <v>0.125</v>
+        <v>0.5</v>
       </c>
       <c r="G24">
         <v>0</v>
@@ -1599,15 +1574,15 @@
         <v>0</v>
       </c>
       <c r="K24" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
     </row>
     <row r="25" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A25" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B25">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="C25" t="s">
         <v>57</v>
@@ -1619,7 +1594,7 @@
         <v>0</v>
       </c>
       <c r="F25" s="1">
-        <v>0.125</v>
+        <v>0.5</v>
       </c>
       <c r="G25">
         <v>0</v>
@@ -1634,15 +1609,15 @@
         <v>0</v>
       </c>
       <c r="K25" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
     </row>
     <row r="26" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A26" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B26">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="C26" t="s">
         <v>57</v>
@@ -1654,7 +1629,7 @@
         <v>0</v>
       </c>
       <c r="F26" s="1">
-        <v>0.125</v>
+        <v>0.5</v>
       </c>
       <c r="G26">
         <v>0</v>
@@ -1669,15 +1644,15 @@
         <v>0</v>
       </c>
       <c r="K26" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
     </row>
     <row r="27" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A27" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B27">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="C27" t="s">
         <v>57</v>
@@ -1689,7 +1664,7 @@
         <v>0</v>
       </c>
       <c r="F27" s="1">
-        <v>1</v>
+        <v>0.5</v>
       </c>
       <c r="G27">
         <v>0</v>
@@ -1704,18 +1679,18 @@
         <v>0</v>
       </c>
       <c r="K27" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
     </row>
     <row r="28" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A28" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B28">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="C28" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="D28" s="1">
         <v>0</v>
@@ -1724,10 +1699,10 @@
         <v>0</v>
       </c>
       <c r="F28" s="1">
-        <v>0</v>
-      </c>
-      <c r="G28" t="s">
-        <v>69</v>
+        <v>0.5</v>
+      </c>
+      <c r="G28">
+        <v>0</v>
       </c>
       <c r="H28">
         <v>0</v>
@@ -1739,15 +1714,15 @@
         <v>0</v>
       </c>
       <c r="K28" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
     </row>
     <row r="29" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A29" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B29">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="C29" t="s">
         <v>58</v>
@@ -1759,10 +1734,10 @@
         <v>0</v>
       </c>
       <c r="F29" s="1">
-        <v>0</v>
-      </c>
-      <c r="G29" t="s">
-        <v>69</v>
+        <v>0.5</v>
+      </c>
+      <c r="G29">
+        <v>8.8499999999999995E-2</v>
       </c>
       <c r="H29">
         <v>0</v>
@@ -1774,15 +1749,15 @@
         <v>0</v>
       </c>
       <c r="K29" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
     </row>
     <row r="30" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A30" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B30">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="C30" t="s">
         <v>58</v>
@@ -1794,10 +1769,10 @@
         <v>0</v>
       </c>
       <c r="F30" s="1">
-        <v>0</v>
-      </c>
-      <c r="G30" t="s">
-        <v>69</v>
+        <v>0.5</v>
+      </c>
+      <c r="G30">
+        <v>8.8499999999999995E-2</v>
       </c>
       <c r="H30">
         <v>0</v>
@@ -1809,15 +1784,15 @@
         <v>0</v>
       </c>
       <c r="K30" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
     </row>
     <row r="31" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A31" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B31">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="C31" t="s">
         <v>58</v>
@@ -1829,10 +1804,10 @@
         <v>0</v>
       </c>
       <c r="F31" s="1">
-        <v>0</v>
-      </c>
-      <c r="G31" t="s">
-        <v>69</v>
+        <v>0.5</v>
+      </c>
+      <c r="G31">
+        <v>8.8499999999999995E-2</v>
       </c>
       <c r="H31">
         <v>0</v>
@@ -1844,15 +1819,15 @@
         <v>0</v>
       </c>
       <c r="K31" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
     </row>
     <row r="32" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A32" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="B32">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="C32" t="s">
         <v>58</v>
@@ -1864,10 +1839,10 @@
         <v>0</v>
       </c>
       <c r="F32" s="1">
-        <v>0</v>
-      </c>
-      <c r="G32" t="s">
-        <v>69</v>
+        <v>0.5</v>
+      </c>
+      <c r="G32">
+        <v>8.8499999999999995E-2</v>
       </c>
       <c r="H32">
         <v>0</v>
@@ -1879,15 +1854,15 @@
         <v>0</v>
       </c>
       <c r="K32" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
     </row>
     <row r="33" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A33" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="B33">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="C33" t="s">
         <v>58</v>
@@ -1899,10 +1874,10 @@
         <v>0</v>
       </c>
       <c r="F33" s="1">
-        <v>0</v>
-      </c>
-      <c r="G33" t="s">
-        <v>69</v>
+        <v>0.5</v>
+      </c>
+      <c r="G33">
+        <v>8.8499999999999995E-2</v>
       </c>
       <c r="H33">
         <v>0</v>
@@ -1914,15 +1889,15 @@
         <v>0</v>
       </c>
       <c r="K33" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
     </row>
     <row r="34" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A34" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="B34">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="C34" t="s">
         <v>58</v>
@@ -1934,10 +1909,10 @@
         <v>0</v>
       </c>
       <c r="F34" s="1">
-        <v>0</v>
-      </c>
-      <c r="G34" t="s">
-        <v>69</v>
+        <v>0.5</v>
+      </c>
+      <c r="G34">
+        <v>8.8499999999999995E-2</v>
       </c>
       <c r="H34">
         <v>0</v>
@@ -1949,15 +1924,15 @@
         <v>0</v>
       </c>
       <c r="K34" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
     </row>
     <row r="35" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A35" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="B35">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="C35" t="s">
         <v>58</v>
@@ -1969,10 +1944,10 @@
         <v>0</v>
       </c>
       <c r="F35" s="1">
-        <v>0</v>
-      </c>
-      <c r="G35" t="s">
-        <v>69</v>
+        <v>0.5</v>
+      </c>
+      <c r="G35">
+        <v>8.8499999999999995E-2</v>
       </c>
       <c r="H35">
         <v>0</v>
@@ -1984,15 +1959,15 @@
         <v>0</v>
       </c>
       <c r="K35" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
     </row>
     <row r="36" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A36" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="B36">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="C36" t="s">
         <v>58</v>
@@ -2004,10 +1979,10 @@
         <v>0</v>
       </c>
       <c r="F36" s="1">
-        <v>0</v>
-      </c>
-      <c r="G36" t="s">
-        <v>69</v>
+        <v>0.5</v>
+      </c>
+      <c r="G36">
+        <v>8.8499999999999995E-2</v>
       </c>
       <c r="H36">
         <v>0</v>
@@ -2019,15 +1994,15 @@
         <v>0</v>
       </c>
       <c r="K36" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
     </row>
     <row r="37" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A37" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="B37">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="C37" t="s">
         <v>58</v>
@@ -2039,10 +2014,10 @@
         <v>0</v>
       </c>
       <c r="F37" s="1">
-        <v>0</v>
-      </c>
-      <c r="G37" t="s">
-        <v>69</v>
+        <v>0.5</v>
+      </c>
+      <c r="G37">
+        <v>8.8499999999999995E-2</v>
       </c>
       <c r="H37">
         <v>0</v>
@@ -2054,15 +2029,15 @@
         <v>0</v>
       </c>
       <c r="K37" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
     </row>
     <row r="38" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A38" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B38">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="C38" t="s">
         <v>58</v>
@@ -2074,10 +2049,10 @@
         <v>0</v>
       </c>
       <c r="F38" s="1">
-        <v>0</v>
-      </c>
-      <c r="G38" t="s">
-        <v>69</v>
+        <v>0.5</v>
+      </c>
+      <c r="G38">
+        <v>8.8499999999999995E-2</v>
       </c>
       <c r="H38">
         <v>0</v>
@@ -2089,15 +2064,15 @@
         <v>0</v>
       </c>
       <c r="K38" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
     </row>
     <row r="39" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A39" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="B39">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C39" t="s">
         <v>58</v>
@@ -2109,10 +2084,10 @@
         <v>0</v>
       </c>
       <c r="F39" s="1">
-        <v>0</v>
-      </c>
-      <c r="G39" t="s">
-        <v>69</v>
+        <v>0.5</v>
+      </c>
+      <c r="G39">
+        <v>8.8499999999999995E-2</v>
       </c>
       <c r="H39">
         <v>0</v>
@@ -2124,15 +2099,15 @@
         <v>0</v>
       </c>
       <c r="K39" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
     </row>
     <row r="40" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A40" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B40">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C40" t="s">
         <v>58</v>
@@ -2144,10 +2119,10 @@
         <v>0</v>
       </c>
       <c r="F40" s="1">
-        <v>0</v>
-      </c>
-      <c r="G40" t="s">
-        <v>69</v>
+        <v>0.5</v>
+      </c>
+      <c r="G40">
+        <v>8.8499999999999995E-2</v>
       </c>
       <c r="H40">
         <v>0</v>
@@ -2159,33 +2134,33 @@
         <v>0</v>
       </c>
       <c r="K40" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
     </row>
     <row r="41" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A41" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="B41">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C41" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="D41" s="1">
         <v>0</v>
       </c>
       <c r="E41" s="1">
-        <v>0.25</v>
+        <v>0</v>
       </c>
       <c r="F41" s="1">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="G41">
-        <v>0</v>
+        <v>8.8499999999999995E-2</v>
       </c>
       <c r="H41">
-        <v>0.25</v>
+        <v>0</v>
       </c>
       <c r="I41">
         <v>0</v>
@@ -2194,15 +2169,15 @@
         <v>0</v>
       </c>
       <c r="K41" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
     </row>
     <row r="42" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A42" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="B42">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C42" t="s">
         <v>59</v>
@@ -2214,7 +2189,7 @@
         <v>0.25</v>
       </c>
       <c r="F42" s="1">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="G42">
         <v>0</v>
@@ -2229,15 +2204,15 @@
         <v>0</v>
       </c>
       <c r="K42" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
     </row>
     <row r="43" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A43" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="B43">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C43" t="s">
         <v>59</v>
@@ -2249,7 +2224,7 @@
         <v>0.25</v>
       </c>
       <c r="F43" s="1">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="G43">
         <v>0</v>
@@ -2264,15 +2239,15 @@
         <v>0</v>
       </c>
       <c r="K43" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
     </row>
     <row r="44" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A44" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="B44">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="C44" t="s">
         <v>59</v>
@@ -2281,16 +2256,16 @@
         <v>0</v>
       </c>
       <c r="E44" s="1">
-        <v>1</v>
+        <v>0.25</v>
       </c>
       <c r="F44" s="1">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="G44">
         <v>0</v>
       </c>
       <c r="H44">
-        <v>1</v>
+        <v>0.25</v>
       </c>
       <c r="I44">
         <v>0</v>
@@ -2299,50 +2274,50 @@
         <v>0</v>
       </c>
       <c r="K44" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
     </row>
     <row r="45" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A45" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="B45">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="C45" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="D45" s="1">
         <v>0</v>
       </c>
       <c r="E45" s="1">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F45" s="1">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="G45">
         <v>0</v>
       </c>
       <c r="H45">
-        <v>0</v>
-      </c>
-      <c r="I45" t="s">
-        <v>67</v>
-      </c>
-      <c r="J45" t="s">
-        <v>67</v>
+        <v>1</v>
+      </c>
+      <c r="I45">
+        <v>0</v>
+      </c>
+      <c r="J45">
+        <v>0</v>
       </c>
       <c r="K45" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
     </row>
     <row r="46" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A46" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="B46">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="C46" t="s">
         <v>60</v>
@@ -2354,7 +2329,7 @@
         <v>0</v>
       </c>
       <c r="F46" s="1">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="G46">
         <v>0</v>
@@ -2362,22 +2337,22 @@
       <c r="H46">
         <v>0</v>
       </c>
-      <c r="I46" t="s">
-        <v>67</v>
-      </c>
-      <c r="J46" t="s">
-        <v>67</v>
+      <c r="I46">
+        <v>9.4E-2</v>
+      </c>
+      <c r="J46">
+        <v>9.4E-2</v>
       </c>
       <c r="K46" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
     </row>
     <row r="47" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A47" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B47">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="C47" t="s">
         <v>60</v>
@@ -2389,7 +2364,7 @@
         <v>0</v>
       </c>
       <c r="F47" s="1">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="G47">
         <v>0</v>
@@ -2397,22 +2372,22 @@
       <c r="H47">
         <v>0</v>
       </c>
-      <c r="I47" t="s">
-        <v>67</v>
-      </c>
-      <c r="J47" t="s">
-        <v>67</v>
+      <c r="I47">
+        <v>9.4E-2</v>
+      </c>
+      <c r="J47">
+        <v>9.4E-2</v>
       </c>
       <c r="K47" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
     </row>
     <row r="48" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A48" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="B48">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="C48" t="s">
         <v>60</v>
@@ -2424,7 +2399,7 @@
         <v>0</v>
       </c>
       <c r="F48" s="1">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="G48">
         <v>0</v>
@@ -2432,22 +2407,22 @@
       <c r="H48">
         <v>0</v>
       </c>
-      <c r="I48" t="s">
-        <v>67</v>
-      </c>
-      <c r="J48" t="s">
-        <v>67</v>
+      <c r="I48">
+        <v>9.4E-2</v>
+      </c>
+      <c r="J48">
+        <v>9.4E-2</v>
       </c>
       <c r="K48" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
     </row>
     <row r="49" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A49" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="B49">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="C49" t="s">
         <v>60</v>
@@ -2459,7 +2434,7 @@
         <v>0</v>
       </c>
       <c r="F49" s="1">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="G49">
         <v>0</v>
@@ -2467,22 +2442,22 @@
       <c r="H49">
         <v>0</v>
       </c>
-      <c r="I49" t="s">
-        <v>67</v>
-      </c>
-      <c r="J49" t="s">
-        <v>67</v>
+      <c r="I49">
+        <v>9.4E-2</v>
+      </c>
+      <c r="J49">
+        <v>9.4E-2</v>
       </c>
       <c r="K49" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
     </row>
     <row r="50" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A50" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="B50">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="C50" t="s">
         <v>60</v>
@@ -2494,7 +2469,7 @@
         <v>0</v>
       </c>
       <c r="F50" s="1">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="G50">
         <v>0</v>
@@ -2502,22 +2477,22 @@
       <c r="H50">
         <v>0</v>
       </c>
-      <c r="I50" t="s">
-        <v>67</v>
-      </c>
-      <c r="J50" t="s">
-        <v>67</v>
+      <c r="I50">
+        <v>9.4E-2</v>
+      </c>
+      <c r="J50">
+        <v>9.4E-2</v>
       </c>
       <c r="K50" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
     </row>
     <row r="51" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A51" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="B51">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="C51" t="s">
         <v>60</v>
@@ -2529,7 +2504,7 @@
         <v>0</v>
       </c>
       <c r="F51" s="1">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="G51">
         <v>0</v>
@@ -2537,22 +2512,22 @@
       <c r="H51">
         <v>0</v>
       </c>
-      <c r="I51" t="s">
-        <v>67</v>
-      </c>
-      <c r="J51" t="s">
-        <v>67</v>
+      <c r="I51">
+        <v>9.4E-2</v>
+      </c>
+      <c r="J51">
+        <v>9.4E-2</v>
       </c>
       <c r="K51" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
     </row>
     <row r="52" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A52" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="B52">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="C52" t="s">
         <v>60</v>
@@ -2564,7 +2539,7 @@
         <v>0</v>
       </c>
       <c r="F52" s="1">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="G52">
         <v>0</v>
@@ -2572,22 +2547,22 @@
       <c r="H52">
         <v>0</v>
       </c>
-      <c r="I52" t="s">
-        <v>67</v>
-      </c>
-      <c r="J52" t="s">
-        <v>67</v>
+      <c r="I52">
+        <v>9.4E-2</v>
+      </c>
+      <c r="J52">
+        <v>9.4E-2</v>
       </c>
       <c r="K52" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
     </row>
     <row r="53" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A53" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B53">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="C53" t="s">
         <v>60</v>
@@ -2599,7 +2574,7 @@
         <v>0</v>
       </c>
       <c r="F53" s="1">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="G53">
         <v>0</v>
@@ -2607,14 +2582,49 @@
       <c r="H53">
         <v>0</v>
       </c>
-      <c r="I53" t="s">
-        <v>67</v>
-      </c>
-      <c r="J53" t="s">
-        <v>67</v>
+      <c r="I53">
+        <v>9.4E-2</v>
+      </c>
+      <c r="J53">
+        <v>9.4E-2</v>
       </c>
       <c r="K53" t="s">
-        <v>71</v>
+        <v>70</v>
+      </c>
+    </row>
+    <row r="54" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A54" t="s">
+        <v>54</v>
+      </c>
+      <c r="B54">
+        <v>52</v>
+      </c>
+      <c r="C54" t="s">
+        <v>60</v>
+      </c>
+      <c r="D54" s="1">
+        <v>0</v>
+      </c>
+      <c r="E54" s="1">
+        <v>0</v>
+      </c>
+      <c r="F54" s="1">
+        <v>0.5</v>
+      </c>
+      <c r="G54">
+        <v>0</v>
+      </c>
+      <c r="H54">
+        <v>0</v>
+      </c>
+      <c r="I54">
+        <v>9.4E-2</v>
+      </c>
+      <c r="J54">
+        <v>9.4E-2</v>
+      </c>
+      <c r="K54" t="s">
+        <v>70</v>
       </c>
     </row>
   </sheetData>

</xml_diff>